<commit_message>
Finalize HS summary MRKU2714799: computed values, notes on COO and HS discrepancy
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JMNoKgzWJHLBkkHVS5evzi
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Ardea_cz_MRKU2714799.xlsx
+++ b/output/HS_Code_Summary_Ardea_cz_MRKU2714799.xlsx
@@ -623,21 +623,17 @@
           <t>Kovové komponenty pro zásuvky do kuchyně / Příslušenství pro kovové zásuvky do kuchyně</t>
         </is>
       </c>
-      <c r="D5" s="7">
-        <f>SUMIFS('Line items'!J$2:J$82,'Line items'!D$2:D$82,B5)</f>
-        <v/>
-      </c>
-      <c r="E5" s="7">
-        <f>SUMIFS('Line items'!K$2:K$82,'Line items'!D$2:D$82,B5)</f>
-        <v/>
-      </c>
-      <c r="F5" s="4">
-        <f>SUMIFS('Line items'!F$2:F$82,'Line items'!D$2:D$82,B5)</f>
-        <v/>
-      </c>
-      <c r="G5" s="8">
-        <f>SUMIFS('Line items'!M$2:M$82,'Line items'!D$2:D$82,B5)</f>
-        <v/>
+      <c r="D5" s="7" t="n">
+        <v>22307.35</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>23245.65</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>14432</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>58161.75</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -666,21 +662,17 @@
           <t>Krytky plastové na bok kovových zásuvek do kuchyně / Plastový profil pro výrobu oddělovačů a příborníků na míru / Plastové koše na prádlo včetně všech dalších věcí / Odpadkový plastový koš do skříňky / Plastový příborník</t>
         </is>
       </c>
-      <c r="D6" s="7">
-        <f>SUMIFS('Line items'!J$2:J$82,'Line items'!D$2:D$82,B6)</f>
-        <v/>
-      </c>
-      <c r="E6" s="7">
-        <f>SUMIFS('Line items'!K$2:K$82,'Line items'!D$2:D$82,B6)</f>
-        <v/>
-      </c>
-      <c r="F6" s="4">
-        <f>SUMIFS('Line items'!F$2:F$82,'Line items'!D$2:D$82,B6)</f>
-        <v/>
-      </c>
-      <c r="G6" s="8">
-        <f>SUMIFS('Line items'!M$2:M$82,'Line items'!D$2:D$82,B6)</f>
-        <v/>
+      <c r="D6" s="7" t="n">
+        <v>1740.589</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>2015.889</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>7834.03</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -701,21 +693,17 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D7" s="10">
-        <f>SUM(D5:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="10">
-        <f>SUM(E5:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="9">
-        <f>SUM(F5:F6)</f>
-        <v/>
-      </c>
-      <c r="G7" s="11">
-        <f>SUM(G5:G6)</f>
-        <v/>
+      <c r="D7" s="10" t="n">
+        <v>24047.939</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>25261.539</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>16792</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>65995.78</v>
       </c>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
@@ -727,14 +715,14 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
           <t>⚠ COO / PREFERENČNÍ VĚTA: NOT present. Invoice and packing list state only 'WE HEREBY CERTIFY THAT THE ABOVE MENTIONED GOODS ARE OF CHINESE ORIGIN.' No preferential-origin declaration (none exists for China–EU) → standard third-country duty applies.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
           <t>⚠ HS DISCREPANCY: Items HC1301W / HC1311W (plastic side caps, 2×500 pcs, EUR 137.00) are 830242 on the invoice/packing list but 3924900090 in the client CSV. This summary follows the client CSV (plastic goods → 3924900090). Confirm before clearance.</t>
@@ -751,14 +739,14 @@
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>Note: Handling fee EUR 114.00 distributed proportionally by value into customs values (8302420090: +100.47 → 58 161.75 · 3924900090: +13.53 → 7 834.03).</t>
+          <t>Note: Handling fee EUR 114.00 distributed proportionally by value into customs values (8302420090: +100.47 -&gt; 58 161.75 · 3924900090: +13.53 -&gt; 7 834.03).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Note: CI line 76 (YG038.60DG) printed value EUR 365.10 differs from unit price × qty (EUR 365.20) by EUR 0.10; invoice printed value used.</t>
+          <t>Note: CI line 76 (YG038.60DG) printed value EUR 365.10 differs from unit price x qty (EUR 365.20) by EUR 0.10; invoice printed value used.</t>
         </is>
       </c>
     </row>
@@ -917,13 +905,11 @@
       <c r="K2" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="L2" s="19">
-        <f>I2/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M2" s="19">
-        <f>I2+L2</f>
-        <v/>
+      <c r="L2" s="19" t="n">
+        <v>0.7030999999999999</v>
+      </c>
+      <c r="M2" s="19" t="n">
+        <v>407.0231</v>
       </c>
     </row>
     <row r="3">
@@ -970,13 +956,11 @@
       <c r="K3" s="22" t="n">
         <v>300</v>
       </c>
-      <c r="L3" s="23">
-        <f>I3/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M3" s="23">
-        <f>I3+L3</f>
-        <v/>
+      <c r="L3" s="23" t="n">
+        <v>1.4062</v>
+      </c>
+      <c r="M3" s="23" t="n">
+        <v>814.0462</v>
       </c>
     </row>
     <row r="4">
@@ -1023,13 +1007,11 @@
       <c r="K4" s="18" t="n">
         <v>167</v>
       </c>
-      <c r="L4" s="19">
-        <f>I4/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M4" s="19">
-        <f>I4+L4</f>
-        <v/>
+      <c r="L4" s="19" t="n">
+        <v>0.7376</v>
+      </c>
+      <c r="M4" s="19" t="n">
+        <v>426.9776</v>
       </c>
     </row>
     <row r="5">
@@ -1076,13 +1058,11 @@
       <c r="K5" s="22" t="n">
         <v>334</v>
       </c>
-      <c r="L5" s="23">
-        <f>I5/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M5" s="23">
-        <f>I5+L5</f>
-        <v/>
+      <c r="L5" s="23" t="n">
+        <v>1.4751</v>
+      </c>
+      <c r="M5" s="23" t="n">
+        <v>853.9551</v>
       </c>
     </row>
     <row r="6">
@@ -1129,13 +1109,11 @@
       <c r="K6" s="18" t="n">
         <v>183</v>
       </c>
-      <c r="L6" s="19">
-        <f>I6/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M6" s="19">
-        <f>I6+L6</f>
-        <v/>
+      <c r="L6" s="19" t="n">
+        <v>0.7652</v>
+      </c>
+      <c r="M6" s="19" t="n">
+        <v>442.9652</v>
       </c>
     </row>
     <row r="7">
@@ -1182,13 +1160,11 @@
       <c r="K7" s="22" t="n">
         <v>366</v>
       </c>
-      <c r="L7" s="23">
-        <f>I7/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M7" s="23">
-        <f>I7+L7</f>
-        <v/>
+      <c r="L7" s="23" t="n">
+        <v>1.5303</v>
+      </c>
+      <c r="M7" s="23" t="n">
+        <v>885.9303</v>
       </c>
     </row>
     <row r="8">
@@ -1235,13 +1211,11 @@
       <c r="K8" s="18" t="n">
         <v>197</v>
       </c>
-      <c r="L8" s="19">
-        <f>I8/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M8" s="19">
-        <f>I8+L8</f>
-        <v/>
+      <c r="L8" s="19" t="n">
+        <v>0.7684</v>
+      </c>
+      <c r="M8" s="19" t="n">
+        <v>444.8284</v>
       </c>
     </row>
     <row r="9">
@@ -1288,13 +1262,11 @@
       <c r="K9" s="22" t="n">
         <v>295.5</v>
       </c>
-      <c r="L9" s="23">
-        <f>I9/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M9" s="23">
-        <f>I9+L9</f>
-        <v/>
+      <c r="L9" s="23" t="n">
+        <v>1.1526</v>
+      </c>
+      <c r="M9" s="23" t="n">
+        <v>667.2426</v>
       </c>
     </row>
     <row r="10">
@@ -1341,13 +1313,11 @@
       <c r="K10" s="18" t="n">
         <v>884</v>
       </c>
-      <c r="L10" s="19">
-        <f>I10/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M10" s="19">
-        <f>I10+L10</f>
-        <v/>
+      <c r="L10" s="19" t="n">
+        <v>3.2035</v>
+      </c>
+      <c r="M10" s="19" t="n">
+        <v>1854.5635</v>
       </c>
     </row>
     <row r="11">
@@ -1394,13 +1364,11 @@
       <c r="K11" s="22" t="n">
         <v>114.1</v>
       </c>
-      <c r="L11" s="23">
-        <f>I11/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M11" s="23">
-        <f>I11+L11</f>
-        <v/>
+      <c r="L11" s="23" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="M11" s="23" t="n">
+        <v>322.445</v>
       </c>
     </row>
     <row r="12">
@@ -1447,13 +1415,11 @@
       <c r="K12" s="18" t="n">
         <v>407.5</v>
       </c>
-      <c r="L12" s="19">
-        <f>I12/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M12" s="19">
-        <f>I12+L12</f>
-        <v/>
+      <c r="L12" s="19" t="n">
+        <v>1.9892</v>
+      </c>
+      <c r="M12" s="19" t="n">
+        <v>1151.5892</v>
       </c>
     </row>
     <row r="13">
@@ -1500,13 +1466,11 @@
       <c r="K13" s="22" t="n">
         <v>184</v>
       </c>
-      <c r="L13" s="23">
-        <f>I13/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M13" s="23">
-        <f>I13+L13</f>
-        <v/>
+      <c r="L13" s="23" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="M13" s="23" t="n">
+        <v>480.47</v>
       </c>
     </row>
     <row r="14">
@@ -1553,13 +1517,11 @@
       <c r="K14" s="18" t="n">
         <v>609</v>
       </c>
-      <c r="L14" s="19">
-        <f>I14/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M14" s="19">
-        <f>I14+L14</f>
-        <v/>
+      <c r="L14" s="19" t="n">
+        <v>2.5721</v>
+      </c>
+      <c r="M14" s="19" t="n">
+        <v>1489.0121</v>
       </c>
     </row>
     <row r="15">
@@ -1606,13 +1568,11 @@
       <c r="K15" s="22" t="n">
         <v>507.5</v>
       </c>
-      <c r="L15" s="23">
-        <f>I15/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M15" s="23">
-        <f>I15+L15</f>
-        <v/>
+      <c r="L15" s="23" t="n">
+        <v>2.1434</v>
+      </c>
+      <c r="M15" s="23" t="n">
+        <v>1240.8434</v>
       </c>
     </row>
     <row r="16">
@@ -1659,13 +1619,11 @@
       <c r="K16" s="18" t="n">
         <v>220</v>
       </c>
-      <c r="L16" s="19">
-        <f>I16/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M16" s="19">
-        <f>I16+L16</f>
-        <v/>
+      <c r="L16" s="19" t="n">
+        <v>0.8721</v>
+      </c>
+      <c r="M16" s="19" t="n">
+        <v>504.8721</v>
       </c>
     </row>
     <row r="17">
@@ -1712,13 +1670,11 @@
       <c r="K17" s="22" t="n">
         <v>488</v>
       </c>
-      <c r="L17" s="23">
-        <f>I17/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M17" s="23">
-        <f>I17+L17</f>
-        <v/>
+      <c r="L17" s="23" t="n">
+        <v>1.8242</v>
+      </c>
+      <c r="M17" s="23" t="n">
+        <v>1056.0242</v>
       </c>
     </row>
     <row r="18">
@@ -1765,13 +1721,11 @@
       <c r="K18" s="18" t="n">
         <v>1220</v>
       </c>
-      <c r="L18" s="19">
-        <f>I18/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M18" s="19">
-        <f>I18+L18</f>
-        <v/>
+      <c r="L18" s="19" t="n">
+        <v>4.5604</v>
+      </c>
+      <c r="M18" s="19" t="n">
+        <v>2640.0604</v>
       </c>
     </row>
     <row r="19">
@@ -1818,13 +1772,11 @@
       <c r="K19" s="22" t="n">
         <v>412.5</v>
       </c>
-      <c r="L19" s="23">
-        <f>I19/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M19" s="23">
-        <f>I19+L19</f>
-        <v/>
+      <c r="L19" s="23" t="n">
+        <v>1.9253</v>
+      </c>
+      <c r="M19" s="23" t="n">
+        <v>1114.5503</v>
       </c>
     </row>
     <row r="20">
@@ -1871,13 +1823,11 @@
       <c r="K20" s="18" t="n">
         <v>412.5</v>
       </c>
-      <c r="L20" s="19">
-        <f>I20/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M20" s="19">
-        <f>I20+L20</f>
-        <v/>
+      <c r="L20" s="19" t="n">
+        <v>1.9253</v>
+      </c>
+      <c r="M20" s="19" t="n">
+        <v>1114.5503</v>
       </c>
     </row>
     <row r="21">
@@ -1924,13 +1874,11 @@
       <c r="K21" s="22" t="n">
         <v>455</v>
       </c>
-      <c r="L21" s="23">
-        <f>I21/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M21" s="23">
-        <f>I21+L21</f>
-        <v/>
+      <c r="L21" s="23" t="n">
+        <v>1.9973</v>
+      </c>
+      <c r="M21" s="23" t="n">
+        <v>1156.2473</v>
       </c>
     </row>
     <row r="22">
@@ -1977,13 +1925,11 @@
       <c r="K22" s="18" t="n">
         <v>455</v>
       </c>
-      <c r="L22" s="19">
-        <f>I22/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M22" s="19">
-        <f>I22+L22</f>
-        <v/>
+      <c r="L22" s="19" t="n">
+        <v>1.9973</v>
+      </c>
+      <c r="M22" s="19" t="n">
+        <v>1156.2473</v>
       </c>
     </row>
     <row r="23">
@@ -2030,13 +1976,11 @@
       <c r="K23" s="22" t="n">
         <v>502.5</v>
       </c>
-      <c r="L23" s="23">
-        <f>I23/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M23" s="23">
-        <f>I23+L23</f>
-        <v/>
+      <c r="L23" s="23" t="n">
+        <v>2.0639</v>
+      </c>
+      <c r="M23" s="23" t="n">
+        <v>1194.8139</v>
       </c>
     </row>
     <row r="24">
@@ -2083,13 +2027,11 @@
       <c r="K24" s="18" t="n">
         <v>502.5</v>
       </c>
-      <c r="L24" s="19">
-        <f>I24/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M24" s="19">
-        <f>I24+L24</f>
-        <v/>
+      <c r="L24" s="19" t="n">
+        <v>2.0639</v>
+      </c>
+      <c r="M24" s="19" t="n">
+        <v>1194.8139</v>
       </c>
     </row>
     <row r="25">
@@ -2136,13 +2078,11 @@
       <c r="K25" s="22" t="n">
         <v>526.25</v>
       </c>
-      <c r="L25" s="23">
-        <f>I25/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M25" s="23">
-        <f>I25+L25</f>
-        <v/>
+      <c r="L25" s="23" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="M25" s="23" t="n">
+        <v>1198.32</v>
       </c>
     </row>
     <row r="26">
@@ -2189,13 +2129,11 @@
       <c r="K26" s="18" t="n">
         <v>631.5</v>
       </c>
-      <c r="L26" s="19">
-        <f>I26/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M26" s="19">
-        <f>I26+L26</f>
-        <v/>
+      <c r="L26" s="19" t="n">
+        <v>2.4839</v>
+      </c>
+      <c r="M26" s="19" t="n">
+        <v>1437.9839</v>
       </c>
     </row>
     <row r="27">
@@ -2242,13 +2180,11 @@
       <c r="K27" s="22" t="n">
         <v>579.25</v>
       </c>
-      <c r="L27" s="23">
-        <f>I27/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M27" s="23">
-        <f>I27+L27</f>
-        <v/>
+      <c r="L27" s="23" t="n">
+        <v>2.1567</v>
+      </c>
+      <c r="M27" s="23" t="n">
+        <v>1248.5317</v>
       </c>
     </row>
     <row r="28">
@@ -2295,13 +2231,11 @@
       <c r="K28" s="18" t="n">
         <v>2548.7</v>
       </c>
-      <c r="L28" s="19">
-        <f>I28/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M28" s="19">
-        <f>I28+L28</f>
-        <v/>
+      <c r="L28" s="19" t="n">
+        <v>9.4894</v>
+      </c>
+      <c r="M28" s="19" t="n">
+        <v>5493.5394</v>
       </c>
     </row>
     <row r="29">
@@ -2348,13 +2282,11 @@
       <c r="K29" s="22" t="n">
         <v>375</v>
       </c>
-      <c r="L29" s="23">
-        <f>I29/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M29" s="23">
-        <f>I29+L29</f>
-        <v/>
+      <c r="L29" s="23" t="n">
+        <v>1.7994</v>
+      </c>
+      <c r="M29" s="23" t="n">
+        <v>1041.6994</v>
       </c>
     </row>
     <row r="30">
@@ -2401,13 +2333,11 @@
       <c r="K30" s="18" t="n">
         <v>435</v>
       </c>
-      <c r="L30" s="19">
-        <f>I30/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M30" s="19">
-        <f>I30+L30</f>
-        <v/>
+      <c r="L30" s="19" t="n">
+        <v>1.8461</v>
+      </c>
+      <c r="M30" s="19" t="n">
+        <v>1068.7461</v>
       </c>
     </row>
     <row r="31">
@@ -2454,13 +2384,11 @@
       <c r="K31" s="22" t="n">
         <v>540</v>
       </c>
-      <c r="L31" s="23">
-        <f>I31/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M31" s="23">
-        <f>I31+L31</f>
-        <v/>
+      <c r="L31" s="23" t="n">
+        <v>2.1807</v>
+      </c>
+      <c r="M31" s="23" t="n">
+        <v>1262.4207</v>
       </c>
     </row>
     <row r="32">
@@ -2507,13 +2435,11 @@
       <c r="K32" s="18" t="n">
         <v>450</v>
       </c>
-      <c r="L32" s="19">
-        <f>I32/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M32" s="19">
-        <f>I32+L32</f>
-        <v/>
+      <c r="L32" s="19" t="n">
+        <v>1.8172</v>
+      </c>
+      <c r="M32" s="19" t="n">
+        <v>1052.0172</v>
       </c>
     </row>
     <row r="33">
@@ -2560,13 +2486,11 @@
       <c r="K33" s="22" t="n">
         <v>696.5</v>
       </c>
-      <c r="L33" s="23">
-        <f>I33/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M33" s="23">
-        <f>I33+L33</f>
-        <v/>
+      <c r="L33" s="23" t="n">
+        <v>2.6558</v>
+      </c>
+      <c r="M33" s="23" t="n">
+        <v>1537.4758</v>
       </c>
     </row>
     <row r="34">
@@ -2613,13 +2537,11 @@
       <c r="K34" s="18" t="n">
         <v>2124</v>
       </c>
-      <c r="L34" s="19">
-        <f>I34/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M34" s="19">
-        <f>I34+L34</f>
-        <v/>
+      <c r="L34" s="19" t="n">
+        <v>7.588</v>
+      </c>
+      <c r="M34" s="19" t="n">
+        <v>4392.788</v>
       </c>
     </row>
     <row r="35">
@@ -2666,13 +2588,11 @@
       <c r="K35" s="22" t="n">
         <v>17</v>
       </c>
-      <c r="L35" s="23">
-        <f>I35/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M35" s="23">
-        <f>I35+L35</f>
-        <v/>
+      <c r="L35" s="23" t="n">
+        <v>0.2185</v>
+      </c>
+      <c r="M35" s="23" t="n">
+        <v>126.5185</v>
       </c>
     </row>
     <row r="36">
@@ -2719,13 +2639,11 @@
       <c r="K36" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="L36" s="19">
-        <f>I36/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M36" s="19">
-        <f>I36+L36</f>
-        <v/>
+      <c r="L36" s="19" t="n">
+        <v>0.2185</v>
+      </c>
+      <c r="M36" s="19" t="n">
+        <v>126.5185</v>
       </c>
     </row>
     <row r="37">
@@ -2772,13 +2690,11 @@
       <c r="K37" s="22" t="n">
         <v>58.8</v>
       </c>
-      <c r="L37" s="23">
-        <f>I37/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M37" s="23">
-        <f>I37+L37</f>
-        <v/>
+      <c r="L37" s="23" t="n">
+        <v>0.3784</v>
+      </c>
+      <c r="M37" s="23" t="n">
+        <v>219.0584</v>
       </c>
     </row>
     <row r="38">
@@ -2825,13 +2741,11 @@
       <c r="K38" s="18" t="n">
         <v>30.3</v>
       </c>
-      <c r="L38" s="19">
-        <f>I38/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M38" s="19">
-        <f>I38+L38</f>
-        <v/>
+      <c r="L38" s="19" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="M38" s="19" t="n">
+        <v>107.105</v>
       </c>
     </row>
     <row r="39">
@@ -2878,13 +2792,11 @@
       <c r="K39" s="22" t="n">
         <v>50.5</v>
       </c>
-      <c r="L39" s="23">
-        <f>I39/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M39" s="23">
-        <f>I39+L39</f>
-        <v/>
+      <c r="L39" s="23" t="n">
+        <v>0.3084</v>
+      </c>
+      <c r="M39" s="23" t="n">
+        <v>178.5084</v>
       </c>
     </row>
     <row r="40">
@@ -2931,13 +2843,11 @@
       <c r="K40" s="18" t="n">
         <v>67.5</v>
       </c>
-      <c r="L40" s="19">
-        <f>I40/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M40" s="19">
-        <f>I40+L40</f>
-        <v/>
+      <c r="L40" s="19" t="n">
+        <v>0.8526</v>
+      </c>
+      <c r="M40" s="19" t="n">
+        <v>493.5526</v>
       </c>
     </row>
     <row r="41">
@@ -2984,13 +2894,11 @@
       <c r="K41" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="L41" s="23">
-        <f>I41/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M41" s="23">
-        <f>I41+L41</f>
-        <v/>
+      <c r="L41" s="23" t="n">
+        <v>0.0339</v>
+      </c>
+      <c r="M41" s="23" t="n">
+        <v>19.6339</v>
       </c>
     </row>
     <row r="42">
@@ -3037,13 +2945,11 @@
       <c r="K42" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L42" s="19">
-        <f>I42/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M42" s="19">
-        <f>I42+L42</f>
-        <v/>
+      <c r="L42" s="19" t="n">
+        <v>0.0339</v>
+      </c>
+      <c r="M42" s="19" t="n">
+        <v>19.6339</v>
       </c>
     </row>
     <row r="43">
@@ -3090,13 +2996,11 @@
       <c r="K43" s="22" t="n">
         <v>12.8</v>
       </c>
-      <c r="L43" s="23">
-        <f>I43/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M43" s="23">
-        <f>I43+L43</f>
-        <v/>
+      <c r="L43" s="23" t="n">
+        <v>0.2074</v>
+      </c>
+      <c r="M43" s="23" t="n">
+        <v>120.0474</v>
       </c>
     </row>
     <row r="44">
@@ -3143,13 +3047,11 @@
       <c r="K44" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="L44" s="19">
-        <f>I44/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M44" s="19">
-        <f>I44+L44</f>
-        <v/>
+      <c r="L44" s="19" t="n">
+        <v>0.2281</v>
+      </c>
+      <c r="M44" s="19" t="n">
+        <v>132.0681</v>
       </c>
     </row>
     <row r="45">
@@ -3196,13 +3098,11 @@
       <c r="K45" s="22" t="n">
         <v>27</v>
       </c>
-      <c r="L45" s="23">
-        <f>I45/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M45" s="23">
-        <f>I45+L45</f>
-        <v/>
+      <c r="L45" s="23" t="n">
+        <v>0.4817</v>
+      </c>
+      <c r="M45" s="23" t="n">
+        <v>278.8817</v>
       </c>
     </row>
     <row r="46">
@@ -3249,13 +3149,11 @@
       <c r="K46" s="18" t="n">
         <v>57</v>
       </c>
-      <c r="L46" s="19">
-        <f>I46/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M46" s="19">
-        <f>I46+L46</f>
-        <v/>
+      <c r="L46" s="19" t="n">
+        <v>0.733</v>
+      </c>
+      <c r="M46" s="19" t="n">
+        <v>424.333</v>
       </c>
     </row>
     <row r="47">
@@ -3302,13 +3200,11 @@
       <c r="K47" s="22" t="n">
         <v>434</v>
       </c>
-      <c r="L47" s="23">
-        <f>I47/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M47" s="23">
-        <f>I47+L47</f>
-        <v/>
+      <c r="L47" s="23" t="n">
+        <v>1.4722</v>
+      </c>
+      <c r="M47" s="23" t="n">
+        <v>852.2722</v>
       </c>
     </row>
     <row r="48">
@@ -3355,13 +3251,11 @@
       <c r="K48" s="18" t="n">
         <v>452</v>
       </c>
-      <c r="L48" s="19">
-        <f>I48/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M48" s="19">
-        <f>I48+L48</f>
-        <v/>
+      <c r="L48" s="19" t="n">
+        <v>1.5319</v>
+      </c>
+      <c r="M48" s="19" t="n">
+        <v>886.8319</v>
       </c>
     </row>
     <row r="49">
@@ -3408,13 +3302,11 @@
       <c r="K49" s="22" t="n">
         <v>337</v>
       </c>
-      <c r="L49" s="23">
-        <f>I49/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M49" s="23">
-        <f>I49+L49</f>
-        <v/>
+      <c r="L49" s="23" t="n">
+        <v>1.0694</v>
+      </c>
+      <c r="M49" s="23" t="n">
+        <v>619.0694</v>
       </c>
     </row>
     <row r="50">
@@ -3461,13 +3353,11 @@
       <c r="K50" s="18" t="n">
         <v>353</v>
       </c>
-      <c r="L50" s="19">
-        <f>I50/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M50" s="19">
-        <f>I50+L50</f>
-        <v/>
+      <c r="L50" s="19" t="n">
+        <v>1.1102</v>
+      </c>
+      <c r="M50" s="19" t="n">
+        <v>642.7102</v>
       </c>
     </row>
     <row r="51">
@@ -3514,13 +3404,11 @@
       <c r="K51" s="22" t="n">
         <v>794</v>
       </c>
-      <c r="L51" s="23">
-        <f>I51/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M51" s="23">
-        <f>I51+L51</f>
-        <v/>
+      <c r="L51" s="23" t="n">
+        <v>2.3512</v>
+      </c>
+      <c r="M51" s="23" t="n">
+        <v>1361.1512</v>
       </c>
     </row>
     <row r="52">
@@ -3567,13 +3455,11 @@
       <c r="K52" s="18" t="n">
         <v>610</v>
       </c>
-      <c r="L52" s="19">
-        <f>I52/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M52" s="19">
-        <f>I52+L52</f>
-        <v/>
+      <c r="L52" s="19" t="n">
+        <v>1.8833</v>
+      </c>
+      <c r="M52" s="19" t="n">
+        <v>1090.2833</v>
       </c>
     </row>
     <row r="53">
@@ -3620,13 +3506,11 @@
       <c r="K53" s="22" t="n">
         <v>285.45</v>
       </c>
-      <c r="L53" s="23">
-        <f>I53/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M53" s="23">
-        <f>I53+L53</f>
-        <v/>
+      <c r="L53" s="23" t="n">
+        <v>6.4505</v>
+      </c>
+      <c r="M53" s="23" t="n">
+        <v>3734.2505</v>
       </c>
     </row>
     <row r="54">
@@ -3673,13 +3557,11 @@
       <c r="K54" s="18" t="n">
         <v>304</v>
       </c>
-      <c r="L54" s="19">
-        <f>I54/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M54" s="19">
-        <f>I54+L54</f>
-        <v/>
+      <c r="L54" s="19" t="n">
+        <v>2.1206</v>
+      </c>
+      <c r="M54" s="19" t="n">
+        <v>1227.6206</v>
       </c>
     </row>
     <row r="55">
@@ -3726,13 +3608,11 @@
       <c r="K55" s="22" t="n">
         <v>40.5</v>
       </c>
-      <c r="L55" s="23">
-        <f>I55/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M55" s="23">
-        <f>I55+L55</f>
-        <v/>
+      <c r="L55" s="23" t="n">
+        <v>0.5054</v>
+      </c>
+      <c r="M55" s="23" t="n">
+        <v>292.5854</v>
       </c>
     </row>
     <row r="56">
@@ -3779,13 +3659,11 @@
       <c r="K56" s="18" t="n">
         <v>40.5</v>
       </c>
-      <c r="L56" s="19">
-        <f>I56/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M56" s="19">
-        <f>I56+L56</f>
-        <v/>
+      <c r="L56" s="19" t="n">
+        <v>0.5054</v>
+      </c>
+      <c r="M56" s="19" t="n">
+        <v>292.5854</v>
       </c>
     </row>
     <row r="57">
@@ -3832,13 +3710,11 @@
       <c r="K57" s="22" t="n">
         <v>5.2</v>
       </c>
-      <c r="L57" s="23">
-        <f>I57/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M57" s="23">
-        <f>I57+L57</f>
-        <v/>
+      <c r="L57" s="23" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="M57" s="23" t="n">
+        <v>31.855</v>
       </c>
     </row>
     <row r="58">
@@ -3885,13 +3761,11 @@
       <c r="K58" s="18" t="n">
         <v>5.2</v>
       </c>
-      <c r="L58" s="19">
-        <f>I58/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M58" s="19">
-        <f>I58+L58</f>
-        <v/>
+      <c r="L58" s="19" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="M58" s="19" t="n">
+        <v>31.855</v>
       </c>
     </row>
     <row r="59">
@@ -3938,13 +3812,11 @@
       <c r="K59" s="22" t="n">
         <v>14.4</v>
       </c>
-      <c r="L59" s="23">
-        <f>I59/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M59" s="23">
-        <f>I59+L59</f>
-        <v/>
+      <c r="L59" s="23" t="n">
+        <v>0.1374</v>
+      </c>
+      <c r="M59" s="23" t="n">
+        <v>79.53740000000001</v>
       </c>
     </row>
     <row r="60">
@@ -3991,13 +3863,11 @@
       <c r="K60" s="18" t="n">
         <v>14.4</v>
       </c>
-      <c r="L60" s="19">
-        <f>I60/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M60" s="19">
-        <f>I60+L60</f>
-        <v/>
+      <c r="L60" s="19" t="n">
+        <v>0.1374</v>
+      </c>
+      <c r="M60" s="19" t="n">
+        <v>79.53740000000001</v>
       </c>
     </row>
     <row r="61">
@@ -4044,13 +3914,11 @@
       <c r="K61" s="22" t="n">
         <v>79</v>
       </c>
-      <c r="L61" s="23">
-        <f>I61/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M61" s="23">
-        <f>I61+L61</f>
-        <v/>
+      <c r="L61" s="23" t="n">
+        <v>0.2902</v>
+      </c>
+      <c r="M61" s="23" t="n">
+        <v>167.9902</v>
       </c>
     </row>
     <row r="62">
@@ -4097,13 +3965,11 @@
       <c r="K62" s="18" t="n">
         <v>79</v>
       </c>
-      <c r="L62" s="19">
-        <f>I62/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M62" s="19">
-        <f>I62+L62</f>
-        <v/>
+      <c r="L62" s="19" t="n">
+        <v>0.2902</v>
+      </c>
+      <c r="M62" s="19" t="n">
+        <v>167.9902</v>
       </c>
     </row>
     <row r="63">
@@ -4150,13 +4016,11 @@
       <c r="K63" s="22" t="n">
         <v>86.5</v>
       </c>
-      <c r="L63" s="23">
-        <f>I63/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M63" s="23">
-        <f>I63+L63</f>
-        <v/>
+      <c r="L63" s="23" t="n">
+        <v>0.3783</v>
+      </c>
+      <c r="M63" s="23" t="n">
+        <v>218.9783</v>
       </c>
     </row>
     <row r="64">
@@ -4203,13 +4067,11 @@
       <c r="K64" s="18" t="n">
         <v>86.5</v>
       </c>
-      <c r="L64" s="19">
-        <f>I64/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M64" s="19">
-        <f>I64+L64</f>
-        <v/>
+      <c r="L64" s="19" t="n">
+        <v>0.3783</v>
+      </c>
+      <c r="M64" s="19" t="n">
+        <v>218.9783</v>
       </c>
     </row>
     <row r="65">
@@ -4256,13 +4118,11 @@
       <c r="K65" s="22" t="n">
         <v>123.75</v>
       </c>
-      <c r="L65" s="23">
-        <f>I65/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M65" s="23">
-        <f>I65+L65</f>
-        <v/>
+      <c r="L65" s="23" t="n">
+        <v>0.4819</v>
+      </c>
+      <c r="M65" s="23" t="n">
+        <v>278.9819</v>
       </c>
     </row>
     <row r="66">
@@ -4309,13 +4169,11 @@
       <c r="K66" s="18" t="n">
         <v>123.75</v>
       </c>
-      <c r="L66" s="19">
-        <f>I66/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M66" s="19">
-        <f>I66+L66</f>
-        <v/>
+      <c r="L66" s="19" t="n">
+        <v>0.4819</v>
+      </c>
+      <c r="M66" s="19" t="n">
+        <v>278.9819</v>
       </c>
     </row>
     <row r="67">
@@ -4362,13 +4220,11 @@
       <c r="K67" s="22" t="n">
         <v>141.5</v>
       </c>
-      <c r="L67" s="23">
-        <f>I67/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M67" s="23">
-        <f>I67+L67</f>
-        <v/>
+      <c r="L67" s="23" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="M67" s="23" t="n">
+        <v>328.267</v>
       </c>
     </row>
     <row r="68">
@@ -4415,13 +4271,11 @@
       <c r="K68" s="18" t="n">
         <v>141.5</v>
       </c>
-      <c r="L68" s="19">
-        <f>I68/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M68" s="19">
-        <f>I68+L68</f>
-        <v/>
+      <c r="L68" s="19" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="M68" s="19" t="n">
+        <v>328.267</v>
       </c>
     </row>
     <row r="69">
@@ -4468,13 +4322,11 @@
       <c r="K69" s="22" t="n">
         <v>5.2</v>
       </c>
-      <c r="L69" s="23">
-        <f>I69/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M69" s="23">
-        <f>I69+L69</f>
-        <v/>
+      <c r="L69" s="23" t="n">
+        <v>0.0536</v>
+      </c>
+      <c r="M69" s="23" t="n">
+        <v>31.0536</v>
       </c>
     </row>
     <row r="70">
@@ -4521,13 +4373,11 @@
       <c r="K70" s="18" t="n">
         <v>4.6</v>
       </c>
-      <c r="L70" s="19">
-        <f>I70/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M70" s="19">
-        <f>I70+L70</f>
-        <v/>
+      <c r="L70" s="19" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="M70" s="19" t="n">
+        <v>42.273</v>
       </c>
     </row>
     <row r="71">
@@ -4574,13 +4424,11 @@
       <c r="K71" s="22" t="n">
         <v>11.6</v>
       </c>
-      <c r="L71" s="23">
-        <f>I71/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M71" s="23">
-        <f>I71+L71</f>
-        <v/>
+      <c r="L71" s="23" t="n">
+        <v>0.0851</v>
+      </c>
+      <c r="M71" s="23" t="n">
+        <v>49.2851</v>
       </c>
     </row>
     <row r="72">
@@ -4627,13 +4475,11 @@
       <c r="K72" s="18" t="n">
         <v>14.4</v>
       </c>
-      <c r="L72" s="19">
-        <f>I72/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M72" s="19">
-        <f>I72+L72</f>
-        <v/>
+      <c r="L72" s="19" t="n">
+        <v>0.0974</v>
+      </c>
+      <c r="M72" s="19" t="n">
+        <v>56.3974</v>
       </c>
     </row>
     <row r="73">
@@ -4680,13 +4526,11 @@
       <c r="K73" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="L73" s="23">
-        <f>I73/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M73" s="23">
-        <f>I73+L73</f>
-        <v/>
+      <c r="L73" s="23" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="M73" s="23" t="n">
+        <v>67.717</v>
       </c>
     </row>
     <row r="74">
@@ -4733,13 +4577,11 @@
       <c r="K74" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="L74" s="19">
-        <f>I74/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M74" s="19">
-        <f>I74+L74</f>
-        <v/>
+      <c r="L74" s="19" t="n">
+        <v>0.1917</v>
+      </c>
+      <c r="M74" s="19" t="n">
+        <v>110.9917</v>
       </c>
     </row>
     <row r="75">
@@ -4786,13 +4628,11 @@
       <c r="K75" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="L75" s="23">
-        <f>I75/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M75" s="23">
-        <f>I75+L75</f>
-        <v/>
+      <c r="L75" s="23" t="n">
+        <v>0.1185</v>
+      </c>
+      <c r="M75" s="23" t="n">
+        <v>68.6185</v>
       </c>
     </row>
     <row r="76">
@@ -4839,13 +4679,11 @@
       <c r="K76" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L76" s="19">
-        <f>I76/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M76" s="19">
-        <f>I76+L76</f>
-        <v/>
+      <c r="L76" s="19" t="n">
+        <v>0.1185</v>
+      </c>
+      <c r="M76" s="19" t="n">
+        <v>68.6185</v>
       </c>
     </row>
     <row r="77">
@@ -4892,13 +4730,11 @@
       <c r="K77" s="22" t="n">
         <v>57.5</v>
       </c>
-      <c r="L77" s="23">
-        <f>I77/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M77" s="23">
-        <f>I77+L77</f>
-        <v/>
+      <c r="L77" s="23" t="n">
+        <v>0.6318</v>
+      </c>
+      <c r="M77" s="23" t="n">
+        <v>365.7318</v>
       </c>
     </row>
     <row r="78">
@@ -4945,13 +4781,11 @@
       <c r="K78" s="18" t="n">
         <v>230</v>
       </c>
-      <c r="L78" s="19">
-        <f>I78/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M78" s="19">
-        <f>I78+L78</f>
-        <v/>
+      <c r="L78" s="19" t="n">
+        <v>2.4458</v>
+      </c>
+      <c r="M78" s="19" t="n">
+        <v>1415.8958</v>
       </c>
     </row>
     <row r="79">
@@ -4998,13 +4832,11 @@
       <c r="K79" s="22" t="n">
         <v>205</v>
       </c>
-      <c r="L79" s="23">
-        <f>I79/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M79" s="23">
-        <f>I79+L79</f>
-        <v/>
+      <c r="L79" s="23" t="n">
+        <v>1.9858</v>
+      </c>
+      <c r="M79" s="23" t="n">
+        <v>1149.5858</v>
       </c>
     </row>
     <row r="80">
@@ -5051,13 +4883,11 @@
       <c r="K80" s="18" t="n">
         <v>500</v>
       </c>
-      <c r="L80" s="19">
-        <f>I80/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M80" s="19">
-        <f>I80+L80</f>
-        <v/>
+      <c r="L80" s="19" t="n">
+        <v>2.9699</v>
+      </c>
+      <c r="M80" s="19" t="n">
+        <v>1719.3199</v>
       </c>
     </row>
     <row r="81">
@@ -5104,13 +4934,11 @@
       <c r="K81" s="22" t="n">
         <v>1000</v>
       </c>
-      <c r="L81" s="23">
-        <f>I81/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M81" s="23">
-        <f>I81+L81</f>
-        <v/>
+      <c r="L81" s="23" t="n">
+        <v>5.2413</v>
+      </c>
+      <c r="M81" s="23" t="n">
+        <v>3034.2413</v>
       </c>
     </row>
     <row r="82">
@@ -5157,13 +4985,11 @@
       <c r="K82" s="18" t="n">
         <v>17.389</v>
       </c>
-      <c r="L82" s="19">
-        <f>I82/$I$83*$L$83</f>
-        <v/>
-      </c>
-      <c r="M82" s="19">
-        <f>I82+L82</f>
-        <v/>
+      <c r="L82" s="19" t="n">
+        <v>0.0208</v>
+      </c>
+      <c r="M82" s="19" t="n">
+        <v>12.0208</v>
       </c>
     </row>
     <row r="83">
@@ -5176,36 +5002,31 @@
       <c r="C83" s="9" t="n"/>
       <c r="D83" s="9" t="n"/>
       <c r="E83" s="9" t="n"/>
-      <c r="F83" s="9">
-        <f>SUM(F2:F82)</f>
-        <v/>
+      <c r="F83" s="9" t="n">
+        <v>16792</v>
       </c>
       <c r="G83" s="9" t="n"/>
       <c r="H83" s="9" t="n"/>
-      <c r="I83" s="11">
-        <f>SUM(I2:I82)</f>
-        <v/>
-      </c>
-      <c r="J83" s="10">
-        <f>SUM(J2:J82)</f>
-        <v/>
-      </c>
-      <c r="K83" s="10">
-        <f>SUM(K2:K82)</f>
-        <v/>
+      <c r="I83" s="11" t="n">
+        <v>65881.783</v>
+      </c>
+      <c r="J83" s="10" t="n">
+        <v>24047.939</v>
+      </c>
+      <c r="K83" s="10" t="n">
+        <v>25261.539</v>
       </c>
       <c r="L83" s="11" t="n">
         <v>114</v>
       </c>
-      <c r="M83" s="11">
-        <f>I83+L83</f>
-        <v/>
+      <c r="M83" s="11" t="n">
+        <v>65995.783</v>
       </c>
     </row>
     <row r="85">
       <c r="B85" s="12" t="inlineStr">
         <is>
-          <t>Handling fee EUR 114.00 (CI line 'Handling fee') is distributed across line items in proportion to value; grand total matches CI total EUR 65,995.783.</t>
+          <t>Handling fee EUR 114.00 (CI line 'Handling fee') distributed across line items in proportion to value; grand total EUR 65,995.783 matches CI total.</t>
         </is>
       </c>
     </row>

</xml_diff>